<commit_message>
Corrige la correction du module 05 : blocs a ordre libre
Applications 1 a 4 et TP : libelles et montants verifies par bloc
(immobilisations, actif circulant, capitaux propres, dettes, charges et
produits), dans n'importe quel ordre, avec colonnes brut/amortissement/
net et signe libre pour la perte. Totaux, resultat et totaux generaux
verifies aux cellules reelles. Intitule Immobilisations incorporelles
restaure dans l'application 1.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/05-bilan/assets/exercices-excel/app-1.xlsx
+++ b/05-bilan/assets/exercices-excel/app-1.xlsx
@@ -726,6 +726,13 @@
         <v>3</v>
       </c>
     </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="19" t="inlineStr">
+        <is>
+          <t>Immobilisations incorporelles</t>
+        </is>
+      </c>
+    </row>
     <row r="7" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="19" t="s">
         <v>9</v>

</xml_diff>